<commit_message>
feat: add Nomor KK field to training registration forms and validation
</commit_message>
<xml_diff>
--- a/public/template-alumni.xlsx
+++ b/public/template-alumni.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="13">
   <si>
     <t>Isi data pelatihan (nama pelatihan, lembaga, tahun, tanggal) di form website, lalu unggah file ini setelah mengisi baris peserta di bawah.</t>
   </si>
@@ -26,6 +26,10 @@
   </si>
   <si>
     <t>NIK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMOR KK
+(16 digit, sama format dengan NIK)</t>
   </si>
   <si>
     <t>JENIS KELAMIN</t>
@@ -469,22 +473,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,8 +501,9 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -529,8 +534,11 @@
       <c r="J2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="52" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="52" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -561,8 +569,11 @@
       <c r="J3" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -572,7 +583,7 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -581,20 +592,23 @@
       <c r="F4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -604,7 +618,7 @@
       <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -613,20 +627,23 @@
       <c r="F5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -636,7 +653,7 @@
       <c r="C6" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -645,20 +662,23 @@
       <c r="F6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>4</v>
       </c>
@@ -668,7 +688,7 @@
       <c r="C7" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -677,20 +697,23 @@
       <c r="F7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>5</v>
       </c>
@@ -700,7 +723,7 @@
       <c r="C8" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -709,20 +732,23 @@
       <c r="F8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>6</v>
       </c>
@@ -732,7 +758,7 @@
       <c r="C9" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -741,20 +767,23 @@
       <c r="F9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>7</v>
       </c>
@@ -764,7 +793,7 @@
       <c r="C10" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
@@ -773,20 +802,23 @@
       <c r="F10" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>8</v>
       </c>
@@ -796,7 +828,7 @@
       <c r="C11" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
@@ -805,20 +837,23 @@
       <c r="F11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>9</v>
       </c>
@@ -828,7 +863,7 @@
       <c r="C12" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -837,20 +872,23 @@
       <c r="F12" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>10</v>
       </c>
@@ -860,7 +898,7 @@
       <c r="C13" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E13" s="4" t="s">
@@ -869,20 +907,23 @@
       <c r="F13" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>11</v>
       </c>
@@ -892,7 +933,7 @@
       <c r="C14" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
@@ -901,20 +942,23 @@
       <c r="F14" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>12</v>
       </c>
@@ -924,7 +968,7 @@
       <c r="C15" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E15" s="4" t="s">
@@ -933,20 +977,23 @@
       <c r="F15" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>13</v>
       </c>
@@ -956,7 +1003,7 @@
       <c r="C16" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -965,20 +1012,23 @@
       <c r="F16" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>14</v>
       </c>
@@ -988,7 +1038,7 @@
       <c r="C17" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E17" s="4" t="s">
@@ -997,20 +1047,23 @@
       <c r="F17" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>15</v>
       </c>
@@ -1020,7 +1073,7 @@
       <c r="C18" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E18" s="4" t="s">
@@ -1029,20 +1082,23 @@
       <c r="F18" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>16</v>
       </c>
@@ -1052,7 +1108,7 @@
       <c r="C19" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E19" s="4" t="s">
@@ -1061,20 +1117,23 @@
       <c r="F19" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>17</v>
       </c>
@@ -1084,7 +1143,7 @@
       <c r="C20" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E20" s="4" t="s">
@@ -1093,20 +1152,23 @@
       <c r="F20" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>18</v>
       </c>
@@ -1116,7 +1178,7 @@
       <c r="C21" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E21" s="4" t="s">
@@ -1125,20 +1187,23 @@
       <c r="F21" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>19</v>
       </c>
@@ -1148,7 +1213,7 @@
       <c r="C22" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E22" s="4" t="s">
@@ -1157,20 +1222,23 @@
       <c r="F22" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G22" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>20</v>
       </c>
@@ -1180,7 +1248,7 @@
       <c r="C23" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>1</v>
       </c>
       <c r="E23" s="4" t="s">
@@ -1189,22 +1257,25 @@
       <c r="F23" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="J23" s="4" t="s">
+      <c r="G23" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>